<commit_message>
Rozrod klubů: doplnit 13 chybějících prev_club_id (jednoznačná pokračování)
fix_missing_links.py: klub bez prev se shodným clean_name a jediným volným ne-B
předchůdcem v minulé sezóně → doplněn link. Např. 1949/50 Sokol Prostějov,
2017/18 řada klubů ← 2016/17, 2018/19 KLAUS Timber.

Chybějící linky 25→12 (zbytek B-týmy/víceznačné, nehádá se), prev 27115→27128,
řetězů 10107→10094, rozbité 0. Konzervativně bez fuzzy přejmenování.
</commit_message>
<xml_diff>
--- a/data/S1967_68_FINAL.xlsx
+++ b/data/S1967_68_FINAL.xlsx
@@ -25090,6 +25090,11 @@
           <t>L20</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>CLUB_S1966_67_0044</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>Slavoj České Budějovice B (Wiki D42 - registr ustavy 04/2026). B-tym hlavni Motor CB chain. city České Budějovice. || TBD: prev_club_id vymazáno (hub-link, nejisté pokračování) [polish_almanach]</t>

</xml_diff>